<commit_message>
feat: adiciona Display TFT 3.5 Touch e 10 botoes tacteis na planilha de compras
</commit_message>
<xml_diff>
--- a/docs/hardware/compras_rover_reorganizado_atualizado.xlsx
+++ b/docs/hardware/compras_rover_reorganizado_atualizado.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Resumo Geral" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UsinaInfo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Mercado Livre" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Curto Circuito" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo Geral" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UsinaInfo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercado Livre" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curto Circuito" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -789,11 +789,11 @@
     </row>
     <row r="6">
       <c r="B6" s="70">
-        <f>'UsinaInfo'!F19+'Mercado Livre'!F14+'Curto Circuito'!F10</f>
+        <f>'UsinaInfo'!F20+'Mercado Livre'!F14+'Curto Circuito'!F10</f>
         <v/>
       </c>
       <c r="D6" s="70">
-        <f>'UsinaInfo'!G19+'Mercado Livre'!G14+'Curto Circuito'!G10</f>
+        <f>'UsinaInfo'!G20+'Mercado Livre'!G14+'Curto Circuito'!G10</f>
         <v/>
       </c>
       <c r="F6" s="70">
@@ -856,11 +856,11 @@
         <v/>
       </c>
       <c r="E11" s="71">
-        <f>'UsinaInfo'!F19</f>
+        <f>'UsinaInfo'!F20</f>
         <v/>
       </c>
       <c r="F11" s="71">
-        <f>'UsinaInfo'!G19</f>
+        <f>'UsinaInfo'!G20</f>
         <v/>
       </c>
       <c r="G11" s="71">
@@ -991,11 +991,11 @@
         </is>
       </c>
       <c r="D19" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Alta",UsinaInfo!F8:F16)+SUMIF('Mercado Livre'!I8:I11,"Alta",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Alta",'Curto Circuito'!F8:F8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Alta",UsinaInfo!F8:F18)+SUMIF('Mercado Livre'!I8:I11,"Alta",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Alta",'Curto Circuito'!F8:F8)</f>
         <v/>
       </c>
       <c r="E19" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Alta",UsinaInfo!G8:G16)+SUMIF('Mercado Livre'!I8:I11,"Alta",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Alta",'Curto Circuito'!G8:G8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Alta",UsinaInfo!G8:G18)+SUMIF('Mercado Livre'!I8:I11,"Alta",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Alta",'Curto Circuito'!G8:G8)</f>
         <v/>
       </c>
       <c r="F19" s="61">
@@ -1015,11 +1015,11 @@
         </is>
       </c>
       <c r="D20" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Média",UsinaInfo!F8:F16)+SUMIF('Mercado Livre'!I8:I11,"Média",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Média",'Curto Circuito'!F8:F8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Média",UsinaInfo!F8:F18)+SUMIF('Mercado Livre'!I8:I11,"Média",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Média",'Curto Circuito'!F8:F8)</f>
         <v/>
       </c>
       <c r="E20" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Média",UsinaInfo!G8:G16)+SUMIF('Mercado Livre'!I8:I11,"Média",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Média",'Curto Circuito'!G8:G8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Média",UsinaInfo!G8:G18)+SUMIF('Mercado Livre'!I8:I11,"Média",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Média",'Curto Circuito'!G8:G8)</f>
         <v/>
       </c>
       <c r="F20" s="61">
@@ -1039,11 +1039,11 @@
         </is>
       </c>
       <c r="D21" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Baixa",UsinaInfo!F8:F16)+SUMIF('Mercado Livre'!I8:I11,"Baixa",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Baixa",'Curto Circuito'!F8:F8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Baixa",UsinaInfo!F8:F18)+SUMIF('Mercado Livre'!I8:I11,"Baixa",'Mercado Livre'!F8:F11)+SUMIF('Curto Circuito'!I8:I8,"Baixa",'Curto Circuito'!F8:F8)</f>
         <v/>
       </c>
       <c r="E21" s="71">
-        <f>SUMIF(UsinaInfo!I8:I16,"Baixa",UsinaInfo!G8:G16)+SUMIF('Mercado Livre'!I8:I11,"Baixa",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Baixa",'Curto Circuito'!G8:G8)</f>
+        <f>SUMIF(UsinaInfo!I8:I18,"Baixa",UsinaInfo!G8:G18)+SUMIF('Mercado Livre'!I8:I11,"Baixa",'Mercado Livre'!G8:G11)+SUMIF('Curto Circuito'!I8:I8,"Baixa",'Curto Circuito'!G8:G8)</f>
         <v/>
       </c>
       <c r="F21" s="61">
@@ -1137,7 +1137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K28"/>
+  <dimension ref="A2:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>Antena Wi-Fi 2,4GHz 3dBi c/ Pigtail U.FL IPEX1</t>
+          <t>Kit Antena Wi-Fi 2,4GHz 3dBi + Cabo Pigtail U.FL (IPEX1) para SMA Fêmea</t>
         </is>
       </c>
       <c r="D12" s="38" t="n">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K12" s="43" t="inlineStr">
         <is>
-          <t>Wi-Fi 2,4 GHz, não antena 4G. Exige conector U.FL/IPEX1 e seleção RF compatíveis na placa. Sem ganho de vídeo garantido.</t>
+          <t>Kit completo: inclui a antena de 3dBi e o cabo adaptador Pigtail U.FL para rosca SMA fêmea.</t>
         </is>
       </c>
     </row>
@@ -1649,74 +1649,139 @@
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="73" t="n"/>
-      <c r="F17" s="73" t="n"/>
-      <c r="G17" s="73" t="n"/>
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>09989</t>
+        </is>
+      </c>
+      <c r="C17" s="45" t="inlineStr">
+        <is>
+          <t>Display TFT LCD 3,5" SPI Touch Screen com Slot SD (ILI9488)</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="76" t="n">
+        <v>119.6</v>
+      </c>
+      <c r="F17" s="76">
+        <f>ROUND(D17*E17,2)</f>
+        <v/>
+      </c>
+      <c r="G17" s="76">
+        <f>ROUND(F17*(1-$D$5),2)</f>
+        <v/>
+      </c>
+      <c r="H17" s="77" t="inlineStr">
+        <is>
+          <t>Abrir produto</t>
+        </is>
+      </c>
+      <c r="I17" s="50" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J17" s="52" t="inlineStr">
+        <is>
+          <t>Em estoque</t>
+        </is>
+      </c>
+      <c r="K17" s="48" t="inlineStr">
+        <is>
+          <t>Display grande 480x320 com touch screen (XPT2046) e slot MicroSD, lógica nativa 3,3 V via SPI.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="E18" s="73" t="n"/>
-      <c r="F18" s="73" t="n"/>
-      <c r="G18" s="73" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>02989</t>
+        </is>
+      </c>
+      <c r="C18" s="45" t="inlineStr">
+        <is>
+          <t>Push Button Chave Táctil 6x6x5mm (2x Kits com 5 un = 10 botões)</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="76" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="F18" s="76">
+        <f>ROUND(D18*E18,2)</f>
+        <v/>
+      </c>
+      <c r="G18" s="76">
+        <f>ROUND(F18*(1-$D$5),2)</f>
+        <v/>
+      </c>
+      <c r="H18" s="77" t="inlineStr">
+        <is>
+          <t>Abrir produto</t>
+        </is>
+      </c>
+      <c r="I18" s="50" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J18" s="52" t="inlineStr">
+        <is>
+          <t>Em estoque</t>
+        </is>
+      </c>
+      <c r="K18" s="48" t="inlineStr">
+        <is>
+          <t>10 chaves tácteis momentâneas para comandos físicos, reset, calibração e botões de interface.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="E19" s="73" t="n"/>
+      <c r="F19" s="73" t="n"/>
+      <c r="G19" s="73" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Total dos itens cotados (UsinaInfo)</t>
         </is>
       </c>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="78" t="n"/>
-      <c r="F19" s="72">
-        <f>SUM(F8:F16)</f>
-        <v/>
-      </c>
-      <c r="G19" s="72">
-        <f>SUM(G8:G16)</f>
-        <v/>
-      </c>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="31" t="n"/>
-      <c r="C20" s="32" t="inlineStr">
-        <is>
-          <t>Subtotal Prioridade Alta (cotados)</t>
-        </is>
-      </c>
-      <c r="D20" s="31" t="n"/>
-      <c r="E20" s="79" t="n"/>
-      <c r="F20" s="80">
-        <f>SUMIF(I8:I16,"Alta",F8:F16)</f>
-        <v/>
-      </c>
-      <c r="G20" s="80">
-        <f>SUMIF(I8:I16,"Alta",G8:G16)</f>
-        <v/>
-      </c>
-      <c r="H20" s="31" t="n"/>
-      <c r="I20" s="31" t="n"/>
-      <c r="J20" s="31" t="n"/>
-      <c r="K20" s="31" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="78" t="n"/>
+      <c r="F20" s="72">
+        <f>SUM(F8:F18)</f>
+        <v/>
+      </c>
+      <c r="G20" s="72">
+        <f>SUM(G8:G18)</f>
+        <v/>
+      </c>
+      <c r="H20" s="11" t="n"/>
+      <c r="I20" s="11" t="n"/>
+      <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="B21" s="31" t="n"/>
       <c r="C21" s="32" t="inlineStr">
         <is>
-          <t>Subtotal Prioridade Média (cotados)</t>
+          <t>Subtotal Prioridade Alta (cotados)</t>
         </is>
       </c>
       <c r="D21" s="31" t="n"/>
       <c r="E21" s="79" t="n"/>
       <c r="F21" s="80">
-        <f>SUMIF(I8:I16,"Média",F8:F16)</f>
+        <f>SUMIF(I8:I18,"Alta",F8:F18)</f>
         <v/>
       </c>
       <c r="G21" s="80">
-        <f>SUMIF(I8:I16,"Média",G8:G16)</f>
+        <f>SUMIF(I8:I18,"Alta",G8:G18)</f>
         <v/>
       </c>
       <c r="H21" s="31" t="n"/>
@@ -1728,17 +1793,17 @@
       <c r="B22" s="31" t="n"/>
       <c r="C22" s="32" t="inlineStr">
         <is>
-          <t>Subtotal Prioridade Baixa (cotados)</t>
+          <t>Subtotal Prioridade Média (cotados)</t>
         </is>
       </c>
       <c r="D22" s="31" t="n"/>
       <c r="E22" s="79" t="n"/>
       <c r="F22" s="80">
-        <f>SUMIF(I8:I16,"Baixa",F8:F16)</f>
+        <f>SUMIF(I8:I18,"Média",F8:F18)</f>
         <v/>
       </c>
       <c r="G22" s="80">
-        <f>SUMIF(I8:I16,"Baixa",G8:G16)</f>
+        <f>SUMIF(I8:I18,"Média",G8:G18)</f>
         <v/>
       </c>
       <c r="H22" s="31" t="n"/>
@@ -1746,37 +1811,59 @@
       <c r="J22" s="31" t="n"/>
       <c r="K22" s="31" t="n"/>
     </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="B24" s="18" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="32" t="inlineStr">
+        <is>
+          <t>Subtotal Prioridade Baixa (cotados)</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="n"/>
+      <c r="E23" s="79" t="n"/>
+      <c r="F23" s="80">
+        <f>SUMIF(I8:I18,"Baixa",F8:F18)</f>
+        <v/>
+      </c>
+      <c r="G23" s="80">
+        <f>SUMIF(I8:I18,"Baixa",G8:G18)</f>
+        <v/>
+      </c>
+      <c r="H23" s="31" t="n"/>
+      <c r="I23" s="31" t="n"/>
+      <c r="J23" s="31" t="n"/>
+      <c r="K23" s="31" t="n"/>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Notas e Observações:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>• ¹ Desconto à vista de 5% configurável na célula D5. Fretes não inclusos.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Preços dos 8 itens conferidos; sensor DC: valor consultado nesta sessão. Estoque pode mudar.</t>
+          <t>• ¹ Desconto à vista de 5% configurável na célula D5. Fretes não inclusos.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="2" t="inlineStr">
         <is>
+          <t>Preços dos 8 itens conferidos; sensor DC: valor consultado nesta sessão. Estoque pode mudar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
           <t>W5500 e ESP auxiliar ausentes nesta versão; controle futuro precisa de placa disponível no laboratório.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" t="inlineStr">
+    <row r="29">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Thermal pad não consta nesta lista. Verificar espessura e área de contato antes de cotar.</t>
         </is>
@@ -1784,7 +1871,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="I8:I16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I8:I18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Alta,Média,Baixa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1798,6 +1885,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1809,7 +1898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K21"/>
+  <dimension ref="B2:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2166,7 +2255,6 @@
       <c r="J16" s="31" t="n"/>
       <c r="K16" s="31" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="18" t="inlineStr">
         <is>

</xml_diff>